<commit_message>
monthly ingredients: 2026-07-01 (17 ingredients, 8 suppliers)
</commit_message>
<xml_diff>
--- a/reports/원료/2026-07-01_신규원료.xlsx
+++ b/reports/원료/2026-07-01_신규원료.xlsx
@@ -465,16 +465,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="35" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -522,33 +522,33 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>TEGO® Pep 4-Even
-(Oligopeptide-68)</t>
+          <t>SPHINOX® Vively
+(Salicyloyl Phytosphingosine)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>미백/톤업 활성물</t>
+          <t>차세대 스핑고지질 바이오액티브 / 피부 장벽 강화</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>세럼, 에센스, 크림</t>
+          <t>세럼, 에센스, 나이트크림, 리치 모이스처라이저</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>멜라닌 생성 억제, 티로시나제 활성 저해, 피부 밝기 개선, 균일한 피부톤</t>
+          <t>레티놀 동등 항노화 효능·자극 없음; 세라마이드 AP·EOP 증가; 바이오텍 유래; PCHi 2026 론칭</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>0.5–2.0%</t>
+          <t>0.1–1.0%</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Evonik 2026 InCosmetics 발표자료 / evonik.com/care</t>
+          <t>Evonik 2026 PCHi 발표 / evonik.com/care</t>
         </is>
       </c>
     </row>
@@ -560,33 +560,33 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>VARISOFT® EQ 100
-(Quaternium-82)</t>
+          <t>RHEANCE® Soft GO
+(Glycolipids, Glyceryl Oleate, Glycerol)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>모발 컨디셔닝제</t>
+          <t>바이오계면활성제 / 피부 장벽 강화 클렌징</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>헤어트리트먼트, 린스, 마스크</t>
+          <t>클렌징 폼, 바디워시, 샴푸, 페이스 워시</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>손상 모발 복원, 빗질성 개선, 정전기 방지, 지속성 매끄러움</t>
+          <t>지속가능 바이오계면활성제; TEWL 감소; 실리콘 대안; in-cosmetics Global 2026 론칭</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>1.0–3.0%</t>
+          <t>0.2–8.0%</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>Evonik 2025 SCC Annual Meeting / evonik.com</t>
+          <t>Evonik in-cosmetics 2026 / evonik.com</t>
         </is>
       </c>
     </row>
@@ -598,33 +598,33 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Pemulen™ TR-3
-(Acrylates/C10-30 Alkyl Acrylate Crosspolymer)</t>
+          <t>NeoHelix™ Regenerate
+(AI 정밀 합성 펩타이드 복합물)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>유화 안정제/증점제</t>
+          <t>적응형 콜라겐 재생 펩타이드</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>O/W 에멀전, 선케어, 워터리 크림</t>
+          <t>항노화 세럼, 에센스, 크림, 앰플</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>고전해질 내성, 투명 겔 형성, 저점도 안정 에멀전 구현</t>
+          <t>56일 후 손상 콜라겐 41% 감소; 피부 HA 65% 증가; AI·바이오엔지니어링 기반; in-cosmetics 2026</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>0.1–0.5%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>BASF Care Creations 2026 라인업 / care-chemicals.basf.com</t>
+          <t>BASF 2026 in-cosmetics / care-chemicals.basf.com</t>
         </is>
       </c>
     </row>
@@ -636,451 +636,527 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Kolliphor® CS 20
-(Ceteareth-20)</t>
+          <t>SkinNexus™ Collag3n
+(재조합 Collagen III 단편, 효모 발효 유래)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>유화제/가용화제</t>
+          <t>비건 Human-Identical 콜라겐 III 단편</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>클렌저, 토너, 투명 에센스</t>
+          <t>항노화 세럼, 크림, 앰플, 마스크팩</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>PEG-free 대안, 바이오 유래 유화, 피부 유분균형 유지</t>
+          <t>Collagen I +48%, III +82%, V +71% (3D 진피 모델); 비건 100% human-identical; 시장 대비 1/10 농도 동등 효과</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>1.0–4.0%</t>
+          <t>TDS 문의 (타사 대비 1/10 수준)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>BASF Formulators Guide 2026 / care-chemicals.basf.com</t>
+          <t>BASF 2026 Press Release / basf.com</t>
         </is>
       </c>
     </row>
     <row r="6" ht="55" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>DSM-Firmenich</t>
+          <t>BASF Care Creations</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Niacinamide XS™
-(Niacinamide)</t>
+          <t>Plantigenix Bisabolol
+(Bisabolol, 바이오텍 발효)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>미백/항산화 비타민</t>
+          <t>발효 생산 (-)-α-비사볼올 / 진정·브라이트닝</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>세럼, 크림, 앰플</t>
+          <t>민감성 피부 크림, 애프터선, 두피케어</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>COGS 최적화 고순도 나이아신아마이드, 모공 축소, 피지 조절, 장벽 강화</t>
+          <t>재생 가능 탄소 100%; 야생 나무 의존 없음; 최고 순도 (-)-이성질체; 저파네솔</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>2.0–10.0%</t>
+          <t>최대 1.0% (leave-on)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>DSM-Firmenich Beauty 2026 Innovation Brief</t>
+          <t>BASF 2026 in-cosmetics / care-chemicals.basf.com</t>
         </is>
       </c>
     </row>
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>DSM-Firmenich</t>
+          <t>BASF Care Creations</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Alpaflor® Edelweiss CA
-(Leontopodium Alpinum Callus Culture Extract)</t>
+          <t>Aloversil™
+(Hippophae Rhamnoides Kernel Extract...)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>항산화/항염 식물 활성물</t>
+          <t>씨버킷 씨박 유래 천연 펩타이드 / 모발 밀도 개선</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>세럼, 선케어, 아이크림</t>
+          <t>헤어 세럼, 리브온 헤어 트리트먼트</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>UV 유래 산화 스트레스 방어, 세포 재생 촉진, 고산 식물 바이오 유래</t>
+          <t>이중맹검 RCT 60명 4개월: 모발 커버리지·밀도 개선; 업사이클 100% 자연 유래</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>0.5–2.0%</t>
+          <t>약 7% w/w</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>DSM-Firmenich Active Beauty Portfolio 2025-2026</t>
+          <t>BASF 2026 Press Release / basf.com</t>
         </is>
       </c>
     </row>
     <row r="8" ht="55" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Givaudan Active Beauty</t>
+          <t>dsm-firmenich</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Gatuline® Skin-Repair Pro
-(Fagus Sylvatica Bud Extract)</t>
+          <t>EXOVIVE™ LIFT
+(Malus Domestica+Citrus+Carica Papaya Extract)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>피부 재생/장벽 강화</t>
+          <t>식물 유래 엑소좀 복합물 / 피부 탄력·항노화</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>나이트크림, 세럼, 에센스</t>
+          <t>항노화 세럼, 크림, 앰플 (분말형, pH 3–10)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>표피 재생 가속, TEWL 감소, 피부 두께 개선, 너도밤나무 줄기세포 유래</t>
+          <t>2개월 후 탄력 30% 향상; 주름 8년치 감소 상당; 식물 유래 엑소좀 화장품 최초 적용 (in-cosmetics 2026)</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>1.0–3.0%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Givaudan Active Beauty 2026 Catalogue / givaudan.com</t>
+          <t>dsm-firmenich 2026 Press / dsm-firmenich.com</t>
         </is>
       </c>
     </row>
     <row r="9" ht="55" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Givaudan Active Beauty</t>
+          <t>dsm-firmenich</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Sepiwhite™ MSH
-(Undecylenoyl Phenylalanine)</t>
+          <t>PARSOL® Shield
+(Bis-Ethylhexyloxyphenol Methoxyphenyl Triazine)</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>미백/색소침착 개선</t>
+          <t>광대역 UVA+UVB 필터 / 광안정성</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>미백 세럼, 스팟 트리트먼트, BB크림</t>
+          <t>선크림, 선로션, 선스프레이, SPF 데이크림</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>α-MSH 차단으로 멜라닌 생성 억제, 기존 기미·잡티 완화</t>
+          <t>FDA 2026년 최종 승인(25년 만에 첫 신규 선크림 원료); Health Canada 최대 6%; 광안정성 우수</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>1.0–3.0%</t>
+          <t>최대 6.0%</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>Givaudan / SEPPIC 2025 공동 마케팅 자료</t>
+          <t>dsm-firmenich 2026 FDA Press / dsm-firmenich.com</t>
         </is>
       </c>
     </row>
     <row r="10" ht="55" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Lonza / Hallstar</t>
+          <t>dsm-firmenich</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Emollient Ester SG-1
-(Isostearyl Isostearate)</t>
+          <t>GLYCARE® SK COMFORT
+(HMO — Human Milk Oligosaccharide, 발효 유래)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>에몰리언트/텍스처 조절</t>
+          <t>모유 올리고당 / 피부 장벽 강화·민감성 개선</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>선스크린, 파운데이션, 보습크림</t>
+          <t>민감성 피부 데이크림, 모이스처라이저, 앰플, 토너</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>비유성(non-greasy) 매끄러움, 유기 자외선 차단제 용해력 우수, 안정성</t>
+          <t>8주 TEWL 16% 감소; 4주 보습 13% 향상; 홍조 개선; 중국 IECIC 등재 완료</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>2.0–10.0%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Hallstar 2026 Emollient Innovation / hallstar.com</t>
+          <t>dsm-firmenich 2026 / dsm-firmenich.com</t>
         </is>
       </c>
     </row>
     <row r="11" ht="55" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Croda International</t>
+          <t>Givaudan Active Beauty</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Phytessence™ Wakame BG
-(Undaria Pinnatifida Extract)</t>
+          <t>PrimalHyal™ NeuroYouth
+(저분자 HA + 아미노산 복합물, MW 20–50 KDa)</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>보습/항노화 해양 활성물</t>
+          <t>신경 피부 노화(Neuro Skin Ageing) 타겟 항노화</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>앰플, 세럼, 보습크림</t>
+          <t>항노화 세럼, 에센스, 나이트크림, 아이크림</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>히알루로니다제 억제로 HA 보호, 탄력 개선, 해양 바이오 지속가능 원료</t>
+          <t>Neuro Skin Ageing 신규 경로 타겟; 마이크로니들링 호환; in-cosmetics 2026 론칭</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>0.5–2.0%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>Croda 2026 Marine Actives / croda.com/personal-care</t>
+          <t>Givaudan Active Beauty 2026 / givaudan.com</t>
         </is>
       </c>
     </row>
     <row r="12" ht="55" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Croda International</t>
+          <t>Croda Beauty (Sederma)</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Inci Plex™ C
-(Sodium PCA, Sodium Lactate, Arginine…)</t>
+          <t>Malvallin™
+(Malva Verticillata Fruit Extract...)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>NMF 복합 보습 시스템</t>
+          <t>중국 아욱 과실 추출물 / 3D 피부 구조 복원</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>수분크림, 토너, 로션</t>
+          <t>안티에이징 세럼, 크림, 앰플, 마스크</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>NMF 10종 복합, 각질층 수화 지속, 피부 pH 균형 유지</t>
+          <t>표피·진피·피하지방 3개 층 동시 볼륨·탄력·보습 개선; COSMOS Natural; 비건·할랄; IECIC 등재</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>2.0–5.0%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Croda 2025-2026 Moisturisation Portfolio</t>
+          <t>Croda Beauty 2026 / crodabeauty.com</t>
         </is>
       </c>
     </row>
     <row r="13" ht="55" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Ashland Personal Care</t>
+          <t>Croda Beauty (Sederma)</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Escalol™ One
-(Bis-Ethylhexyloxyphenol Methoxyphenyl Triazine)</t>
+          <t>Matrixyl® Neolide™
+(Palmitoyl Pentapeptide-4, 리포좀 캡슐화)</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>자외선 차단 필터</t>
+          <t>차세대 Matrixyl / 15일 지속방출 펩타이드</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>선스크린, 데이크림, 파운데이션</t>
+          <t>항노화 세럼, 크림, 앰플, 마이크로니들링 후처리</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>UVA/UVB 광범위 차단, 광안정성 우수, EU/ASEAN 승인 필터</t>
+          <t>2주 탄력 +25%; 마이크로니들링 병용 Collagen III +31%; 최대 15일 지속 방출</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>0.5–3.0%</t>
+          <t>TDS 문의 (전 세대 Matrixyl 3000: 3% 참고)</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>Ashland 2026 Sun Care Innovation / ashland.com</t>
+          <t>Croda 2026 / croda.com</t>
         </is>
       </c>
     </row>
     <row r="14" ht="55" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Ashland Personal Care</t>
+          <t>Ashland Specialty Ingredients</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Benecel™ MHPC
-(Hydroxypropyl Methylcellulose)</t>
+          <t>eternight™ biofunctional
+(Iris Pallida Root Extract...)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>수용성 증점제/필름형성제</t>
+          <t>미토바이올로지 기반 야간 피부 장수 활성물</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>클렌저, 마스크팩, 젤</t>
+          <t>나이트크림, 나이트세럼, 수면 마스크 (leave-on 야간)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>천연 셀룰로스 유래, 깨끗한 포뮬러링, 비건 인증, 피부 쿨링감</t>
+          <t>1개월 후 AI 분석 4년 젊어진 피부; 미토콘드리아 기능 지지; 재생 농업 프랑스산; PCHi 2026 글로벌 론칭</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>0.5–2.0%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Ashland Cellulosics 2026 / ashland.com/personal-care</t>
+          <t>Ashland 2026 PCHi Press / ashland.com</t>
         </is>
       </c>
     </row>
     <row r="15" ht="55" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>코스맥스</t>
+          <t>Hallstar Beauty</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>COSMAX BIO-LIFT Complex
-(Acetyl Hexapeptide-3, Hyaluronic Acid, Ceramide NP)</t>
+          <t>HallSens™ DIAS
+(Diisoamyl Succinate)</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>항노화 복합 활성물</t>
+          <t>100% 식물 유래 업사이클 에몰리언트</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>리프팅 세럼, 아이크림, 텐션크림</t>
+          <t>페이셜 크림, 메이크업, 선크림, 세럼, 헤어케어 전반</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>SNAP-25 억제 리프팅, 실시간 피부 장력 향상, 24h 보습, K-Beauty 특허</t>
+          <t>67% 이상 업사이클 원료(폐기물 유래); 재생 호박산+이소아밀알코올; 저탄소 발자국; 실키 감촉</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>1.0–3.0%</t>
+          <t>2–10%</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>코스맥스 R&amp;I센터 2026 신원료 발표 / cosmax.co.kr</t>
+          <t>Hallstar 2026 / hallstarbeauty.com</t>
         </is>
       </c>
     </row>
     <row r="16" ht="55" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>한국콜마</t>
+          <t>Hallstar Beauty</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>KOLMAR Phyto-Retinol ACX
-(Bakuchiol, Rosehip Seed Oil, Tocopherol)</t>
+          <t>UBI Oléoactif®
+(Betula Alba Bark Extract, Brassica Campestris Seed Oil...)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>레티놀 대안 항노화</t>
+          <t>유기농 자작나무 껍질 추출물 / 브라이트닝·항노화</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>나이트세럼, 레티놀 크림 대체, 안티에이징 앰플</t>
+          <t>스킨케어 세럼, 오일, 나이트크림 (지용성 제형)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>레티놀 동등 항노화 효능, 자극 최소화, 임산부 사용 가능, 식물 유래 100%</t>
+          <t>프랑스산 유기농 자작나무; Oléo-éco-extraction™ 물리적 공정; 피부 톤 균일화·광채·주름 임상 데이터</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>0.5–2.0%</t>
+          <t>TDS 문의</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>한국콜마 2026 소재연구소 신규 식물성 소재 발표</t>
+          <t>Hallstar 2026 / hallstarbeauty.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="55" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>한국콜마 (Korea Kolmar)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>TOT (Tocopherol-Oxalate-Tocopherol)
+(퍼옥살레이트 링커 토코페롤 이량체)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>H₂O₂ 반응성 표적 항산화 신소재</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>항노화 에센스, 세럼, 크림 (스마트 리포좀 적용)</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>30분 내 H₂O₂ 40% 이상 감소; 비타민 E 1/10 농도로 동등 효과; SCI 국제학술지 Molecules 2026 표지논문</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>일반 비타민 E 대비 1/10 (TDS 미공개)</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>한국콜마 R&amp;D / cosinkorea.com 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="55" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>코스맥스바이오 (Cosmax Bio)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>테올림™ (Theolim™)
+(Key Lime Extract + Cacao Extract)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>키라임+카카오 복합 / 체지방 감소·기능성</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>건강기능식품 (주); 기능성 바디·슬리밍 화장품 연구 중</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>RCT 120명: 체지방 6% 감소; GLP-1 +33%, 아디포넥틴 +54.5%; 식약처 개별인정형 원료 2026년 승인</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>식약처 승인 용량 기준</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>코스맥스바이오 2026 / news1.kr</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1178,7 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="38" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1147,22 +1223,22 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Phytessence™ Wakame BG (Croda)</t>
+          <t>PARSOL® Shield (dsm-firmenich)</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>보습/안티에이징 세럼 라인</t>
+          <t>선케어 프리미엄 라인</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>히알루로니다제 억제로 피부 내 HA 보호 → 기존 HA 세럼과 시너지. 해양 지속가능 원료로 클린뷰티 포지셔닝 강화</t>
+          <t>FDA 25년 만에 첫 승인 신규 UV필터. 광안정성 우수한 UVA·UVB 광대역 차단으로 선케어 신제품 포뮬러 차별화 핵심 원료. 규제 이정표로 마케팅 소재 풍부</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>피부 속 HA 보호, 탄력 개선, 해양 유래 에코 포뮬러</t>
+          <t>FDA 최신 승인 UVA·UVB 광대역 차단, 광안정성 강화 선스크린</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -1179,7 +1255,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>KOLMAR Phyto-Retinol ACX (한국콜마)</t>
+          <t>SPHINOX® Vively — Evonik</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -1189,12 +1265,12 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>레티놀 대안 수요 급증(민감성 소비자). 국내 ODM 소싱으로 리드타임 단축, 임산부·민감성 세그먼트 확대 가능</t>
+          <t>레티놀 대안 수요 폭증 (민감성·임산부 소비자). 자극 없이 레티놀 동등 효능 스핑고지질 — K-Beauty 트렌드 '조용한 레티놀 대안' 에 최적화된 스토리텔링 가능</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>자극없는 레티놀 대안, 주름개선, 임산부 안심 성분</t>
+          <t>자극 없는 레티놀 대안, 세라마이드 강화 피부 장벽, 야간 재생</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -1211,22 +1287,22 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>DSM-Firmenich Alpaflor® Edelweiss CA</t>
+          <t>EXOVIVE™ LIFT (dsm-firmenich)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>선케어 / 고기능 UV 세럼</t>
+          <t>프리미엄 안티에이징 앰플 라인</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>에델바이스 줄기세포 추출물 → 스토리텔링 강점. UV 후 산화 스트레스 케어 컨셉으로 선케어 프리미엄 라인 차별화</t>
+          <t>엑소좀 뷰티 최초 식물 유래 상업화 원료 — 차세대 바이오텍 뷰티 트렌드 선점 가능. 2개월 30% 탄력 향상 임상 데이터로 고가 앰플 론칭 시 강력한 근거 확보</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>UV 산화 스트레스 방어, 고산 식물 에너지, 세포 재생</t>
+          <t>식물 엑소좀 바이오텍 탄력 앰플, 2개월 탄력 30% 향상</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -1243,22 +1319,22 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Gatuline® Skin-Repair Pro (Givaudan)</t>
+          <t>Matrixyl® Neolide™ (Croda Sederma)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>나이트크림 / 집중 재생 라인</t>
+          <t>프리미엄 리프팅·탄력 세럼</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>식물 줄기세포 유래 재생 활성물. 야간 재생 크림 컨셉에 적합, 너도밤나무 바이오 소재로 클린뷰티 어필</t>
+          <t>Matrixyl 30년 브랜드 파워 + 15일 지속방출 신기술. 마이크로니들링 병용 시너지로 뷰티디바이스 트렌드와 연계한 차별화 포지셔닝 가능</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>수면 중 피부 재생, 표피 복원, 식물 줄기세포 케어</t>
+          <t>15일 지속 리프팅, Matrixyl 차세대 기술, 디바이스 시너지</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1275,27 +1351,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>COSMAX BIO-LIFT Complex</t>
+          <t>eternight™ biofunctional (Ashland)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>리프팅 / 텐션케어 라인</t>
+          <t>나이트케어 / 수면 뷰티 라인</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>국내 K-Beauty 특허 원료로 소싱 용이. 펩타이드+HA+세라마이드 복합 → 리프팅 세럼 풀패키지 솔루션</t>
+          <t>수면 뷰티(Sleepmaxxing) 트렌드와 완벽한 부합. AI 분석 '4년 젊어진 피부' 스토리텔링, 재생 농업 원료 지속가능성 메시지 동시 소구 가능</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>즉각 리프팅, 주름개선, 24h 피부 장벽 강화</t>
+          <t>수면 중 미토콘드리아 재생, AI 검증 야간 항노화, 지속가능 원료</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>6개월 내 검토</t>
+          <t>3개월 내 검토</t>
         </is>
       </c>
     </row>
@@ -1307,22 +1383,22 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Escalol™ One (Ashland)</t>
+          <t>한국콜마 TOT 표적 항산화</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>선케어 신제품</t>
+          <t>항산화 / 안티폴루션 라인</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>광안정성 높은 UVA/UVB 필터. 기존 선스크린 포뮬러 고도화 시 핵심 성분으로 활용 가능</t>
+          <t>국내 ODM 소싱 가능으로 리드타임 단축. SCI 논문 기반 학술적 신뢰도 + 비타민 E 1/10 농도 고효율 = 고기능·저자극 포지셔닝. 상용화 초기 선점 기회</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>UVA·UVB 동시 차단, 광안정, PA++++ 등급 포뮬러 구현</t>
+          <t>차세대 표적 항산화, 과산화수소 선택적 제거, 피부 산화 스트레스 방어</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">

</xml_diff>